<commit_message>
Add EY vs JustPlay / Lihuhu comparison sheets to fee workbook
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01MGNZa9FoKJ1mnmQ2XmKaEy
</commit_message>
<xml_diff>
--- a/Scrambly_자문사_보수비교.xlsx
+++ b/Scrambly_자문사_보수비교.xlsx
@@ -8,8 +8,10 @@
   </bookViews>
   <sheets>
     <sheet name="비교표" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="건별 개요" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="전제·팩트체크" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="EY vs JustPlay" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="EY vs Lihuhu" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="건별 개요" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet name="전제·팩트체크" sheetId="5" state="visible" r:id="rId5"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -18,11 +20,12 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="2">
+  <numFmts count="3">
     <numFmt numFmtId="164" formatCode="#,##0.0;[Red]-#,##0.0;&quot;-&quot;"/>
     <numFmt numFmtId="165" formatCode="0.0%;[Red]-0.0%"/>
+    <numFmt numFmtId="166" formatCode="#,##0.0;[Red]-#,##0.0"/>
   </numFmts>
-  <fonts count="9">
+  <fonts count="11">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -56,8 +59,15 @@
       <b val="1"/>
       <sz val="12"/>
     </font>
+    <font>
+      <color rgb="00999999"/>
+    </font>
+    <font>
+      <color rgb="00666666"/>
+      <sz val="9"/>
+    </font>
   </fonts>
-  <fills count="5">
+  <fills count="7">
     <fill>
       <patternFill/>
     </fill>
@@ -77,6 +87,16 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="00D9E1F2"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00F2F2F2"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00FFE699"/>
       </patternFill>
     </fill>
   </fills>
@@ -106,7 +126,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="24">
+  <cellXfs count="31">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -158,6 +178,25 @@
     <xf numFmtId="164" fontId="3" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="164" fontId="3" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="166" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="164" fontId="9" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="164" fontId="3" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="164" fontId="3" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="166" fontId="3" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="6" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center" wrapText="1"/>
     </xf>
@@ -1284,6 +1323,638 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
+  <dimension ref="A1:E20"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="24" customWidth="1" min="1" max="1"/>
+    <col width="20" customWidth="1" min="2" max="2"/>
+    <col width="20" customWidth="1" min="3" max="3"/>
+    <col width="20" customWidth="1" min="4" max="4"/>
+    <col width="16" customWidth="1" min="5" max="5"/>
+    <col width="14" customWidth="1" min="6" max="6"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>[Scrambly] 실사 자문 보수 비교 – EY 제안 vs Deloitte JustPlay</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>단위: 백만원, VAT 제외 / 환율은 '비교표' 시트 B5:B6 연동</t>
+        </is>
+      </c>
+    </row>
+    <row r="4" ht="32" customHeight="1">
+      <c r="A4" s="6" t="inlineStr">
+        <is>
+          <t>항목</t>
+        </is>
+      </c>
+      <c r="B4" s="6" t="inlineStr">
+        <is>
+          <t>EY Scrambly
+(제안)</t>
+        </is>
+      </c>
+      <c r="C4" s="6" t="inlineStr">
+        <is>
+          <t>Deloitte JP
+(제안)</t>
+        </is>
+      </c>
+      <c r="D4" s="6" t="inlineStr">
+        <is>
+          <t>Deloitte JP
+(실제)</t>
+        </is>
+      </c>
+      <c r="E4" s="6" t="inlineStr">
+        <is>
+          <t>EY vs JP 실제</t>
+        </is>
+      </c>
+    </row>
+    <row r="5" ht="30" customHeight="1">
+      <c r="A5" s="23" t="inlineStr">
+        <is>
+          <t>FDD</t>
+        </is>
+      </c>
+      <c r="B5" s="11" t="n">
+        <v>140</v>
+      </c>
+      <c r="C5" s="10" t="n">
+        <v>180</v>
+      </c>
+      <c r="D5" s="10" t="n">
+        <v>162</v>
+      </c>
+      <c r="E5" s="24">
+        <f>TEXT(B5-D5,"+#,##0;-#,##0")&amp;" ("&amp;TEXT(B5/D5-1,"+0%;-0%")&amp;")"</f>
+        <v/>
+      </c>
+    </row>
+    <row r="6" ht="30" customHeight="1">
+      <c r="A6" s="23" t="inlineStr">
+        <is>
+          <t>TDD</t>
+        </is>
+      </c>
+      <c r="B6" s="11" t="n">
+        <v>90</v>
+      </c>
+      <c r="C6" s="10">
+        <f>118000*비교표!$B$6/1000000</f>
+        <v/>
+      </c>
+      <c r="D6" s="10" t="n">
+        <v>191</v>
+      </c>
+      <c r="E6" s="24">
+        <f>TEXT(B6-D6,"+#,##0;-#,##0")&amp;" ("&amp;TEXT(B6/D6-1,"+0%;-0%")&amp;")"</f>
+        <v/>
+      </c>
+    </row>
+    <row r="7" ht="30" customHeight="1">
+      <c r="A7" s="23" t="inlineStr">
+        <is>
+          <t>인수구조 검토</t>
+        </is>
+      </c>
+      <c r="B7" s="11" t="inlineStr">
+        <is>
+          <t>Hourly (EUR 504/h, Cap 없음)</t>
+        </is>
+      </c>
+      <c r="C7" s="10">
+        <f>20000*비교표!$B$6/1000000</f>
+        <v/>
+      </c>
+      <c r="D7" s="25" t="inlineStr">
+        <is>
+          <t>별도 항목 없음</t>
+        </is>
+      </c>
+      <c r="E7" s="24" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="8" ht="30" customHeight="1">
+      <c r="A8" s="23" t="inlineStr">
+        <is>
+          <t>SPA/SHA 자문</t>
+        </is>
+      </c>
+      <c r="B8" s="11" t="inlineStr">
+        <is>
+          <t>Hourly (Cap 5)</t>
+        </is>
+      </c>
+      <c r="C8" s="10" t="inlineStr">
+        <is>
+          <t>Hourly</t>
+        </is>
+      </c>
+      <c r="D8" s="10" t="n">
+        <v>71</v>
+      </c>
+      <c r="E8" s="24" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="9" ht="30" customHeight="1">
+      <c r="A9" s="23" t="inlineStr">
+        <is>
+          <t>ITDD</t>
+        </is>
+      </c>
+      <c r="B9" s="11" t="inlineStr">
+        <is>
+          <t>범위 외</t>
+        </is>
+      </c>
+      <c r="C9" s="10" t="inlineStr">
+        <is>
+          <t>범위 외</t>
+        </is>
+      </c>
+      <c r="D9" s="10" t="n">
+        <v>56</v>
+      </c>
+      <c r="E9" s="24" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="10" ht="30" customHeight="1">
+      <c r="A10" s="23" t="inlineStr">
+        <is>
+          <t>기타 실비</t>
+        </is>
+      </c>
+      <c r="B10" s="11" t="inlineStr">
+        <is>
+          <t>별도</t>
+        </is>
+      </c>
+      <c r="C10" s="10" t="inlineStr">
+        <is>
+          <t>별도</t>
+        </is>
+      </c>
+      <c r="D10" s="10" t="n">
+        <v>6</v>
+      </c>
+      <c r="E10" s="24" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="11" ht="30" customHeight="1">
+      <c r="A11" s="26" t="inlineStr">
+        <is>
+          <t>합계 (VAT 제외)</t>
+        </is>
+      </c>
+      <c r="B11" s="27" t="inlineStr">
+        <is>
+          <t>230 + α</t>
+        </is>
+      </c>
+      <c r="C11" s="13">
+        <f>C5+C6</f>
+        <v/>
+      </c>
+      <c r="D11" s="13">
+        <f>SUM(D5:D10)</f>
+        <v/>
+      </c>
+      <c r="E11" s="28" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="12" ht="30" customHeight="1">
+      <c r="A12" s="26" t="inlineStr">
+        <is>
+          <t>FDD+TDD (동일 범위)</t>
+        </is>
+      </c>
+      <c r="B12" s="27">
+        <f>B5+B6</f>
+        <v/>
+      </c>
+      <c r="C12" s="13">
+        <f>C5+C6</f>
+        <v/>
+      </c>
+      <c r="D12" s="13">
+        <f>D5+D6</f>
+        <v/>
+      </c>
+      <c r="E12" s="28">
+        <f>TEXT(B12-D12,"+#,##0;-#,##0")&amp;" ("&amp;TEXT(B12/D12-1,"+0%;-0%")&amp;")"</f>
+        <v/>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>• FDD: JP 실제는 제안 대비 정확히 10% 할인 (180 → 162)</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>• TDD: JP는 독일 2 + 키프로스 1 = 3개 법인 (법인당 ≈64) → 단순 비교 시 차이 과대</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>• JP 총액은 제안 ≈375 → 실제 486 (+30%): ITDD 56, SPA/SHA 71 추가 발생</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>• EY도 SPA·세무 Hourly·실비 추가 시 VAT 포함 약 260~300 예상(추정) → 세무 Hourly Cap 협의 필요</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>• 투입인력: EY 한국 FT 2명 + 파트너·이사, Italy Senior 1명 (4주) vs JP FT 5명 + PT 2명 (4~5주)</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="29" t="inlineStr">
+        <is>
+          <t>※ JP 실제 VAT 포함 535 (지출결의서 20260616-00279) / 출처: EY 제안서 p.20, Deloitte 제안서(260130) p.27</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:E21"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="24" customWidth="1" min="1" max="1"/>
+    <col width="20" customWidth="1" min="2" max="2"/>
+    <col width="20" customWidth="1" min="3" max="3"/>
+    <col width="20" customWidth="1" min="4" max="4"/>
+    <col width="16" customWidth="1" min="5" max="5"/>
+    <col width="14" customWidth="1" min="6" max="6"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>[Scrambly] 실사 자문 보수 비교 – EY 제안 vs Deloitte Lihuhu</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>단위: 백만원, VAT 제외 / 환율은 '비교표' 시트 B5:B6 연동</t>
+        </is>
+      </c>
+    </row>
+    <row r="4" ht="32" customHeight="1">
+      <c r="A4" s="6" t="inlineStr">
+        <is>
+          <t>항목</t>
+        </is>
+      </c>
+      <c r="B4" s="6" t="inlineStr">
+        <is>
+          <t>EY Scrambly
+(제안)</t>
+        </is>
+      </c>
+      <c r="C4" s="6" t="inlineStr">
+        <is>
+          <t>Deloitte Lihuhu
+(제안)</t>
+        </is>
+      </c>
+      <c r="D4" s="6" t="inlineStr">
+        <is>
+          <t>Deloitte Lihuhu
+(실제)</t>
+        </is>
+      </c>
+      <c r="E4" s="6" t="inlineStr">
+        <is>
+          <t>EY vs Lihuhu 제안</t>
+        </is>
+      </c>
+    </row>
+    <row r="5" ht="30" customHeight="1">
+      <c r="A5" s="23" t="inlineStr">
+        <is>
+          <t>FDD</t>
+        </is>
+      </c>
+      <c r="B5" s="11" t="n">
+        <v>140</v>
+      </c>
+      <c r="C5" s="10" t="n">
+        <v>216</v>
+      </c>
+      <c r="D5" s="25" t="inlineStr">
+        <is>
+          <t>항목별 내역 없음</t>
+        </is>
+      </c>
+      <c r="E5" s="24">
+        <f>TEXT(B5-C5,"+#,##0;-#,##0")&amp;" ("&amp;TEXT(B5/C5-1,"+0%;-0%")&amp;")"&amp;" *가치평가 포함"</f>
+        <v/>
+      </c>
+    </row>
+    <row r="6" ht="30" customHeight="1">
+      <c r="A6" s="23" t="inlineStr">
+        <is>
+          <t>가치평가</t>
+        </is>
+      </c>
+      <c r="B6" s="11" t="inlineStr">
+        <is>
+          <t>범위 외</t>
+        </is>
+      </c>
+      <c r="C6" s="10" t="inlineStr">
+        <is>
+          <t>FDD에 포함</t>
+        </is>
+      </c>
+      <c r="D6" s="25" t="inlineStr">
+        <is>
+          <t>항목별 내역 없음</t>
+        </is>
+      </c>
+      <c r="E6" s="24" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="7" ht="30" customHeight="1">
+      <c r="A7" s="23" t="inlineStr">
+        <is>
+          <t>TDD</t>
+        </is>
+      </c>
+      <c r="B7" s="11" t="n">
+        <v>90</v>
+      </c>
+      <c r="C7" s="10">
+        <f>46000*비교표!$B$5/1000000</f>
+        <v/>
+      </c>
+      <c r="D7" s="25" t="inlineStr">
+        <is>
+          <t>항목별 내역 없음</t>
+        </is>
+      </c>
+      <c r="E7" s="24">
+        <f>TEXT(B7-C7,"+#,##0;-#,##0")&amp;" ("&amp;TEXT(B7/C7-1,"+0%;-0%")&amp;")"</f>
+        <v/>
+      </c>
+    </row>
+    <row r="8" ht="30" customHeight="1">
+      <c r="A8" s="23" t="inlineStr">
+        <is>
+          <t>인수구조 검토</t>
+        </is>
+      </c>
+      <c r="B8" s="11" t="inlineStr">
+        <is>
+          <t>Hourly (EUR 504/h, Cap 없음)</t>
+        </is>
+      </c>
+      <c r="C8" s="10">
+        <f>50000*비교표!$B$5/1000000</f>
+        <v/>
+      </c>
+      <c r="D8" s="25" t="inlineStr">
+        <is>
+          <t>결의서 미기재</t>
+        </is>
+      </c>
+      <c r="E8" s="24" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="9" ht="30" customHeight="1">
+      <c r="A9" s="23" t="inlineStr">
+        <is>
+          <t>SPA/SHA 자문</t>
+        </is>
+      </c>
+      <c r="B9" s="11" t="inlineStr">
+        <is>
+          <t>Hourly (Cap 5)</t>
+        </is>
+      </c>
+      <c r="C9" s="10" t="inlineStr">
+        <is>
+          <t>Hourly</t>
+        </is>
+      </c>
+      <c r="D9" s="25" t="inlineStr">
+        <is>
+          <t>결의서 미기재</t>
+        </is>
+      </c>
+      <c r="E9" s="24" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="10" ht="30" customHeight="1">
+      <c r="A10" s="23" t="inlineStr">
+        <is>
+          <t>기타 실비</t>
+        </is>
+      </c>
+      <c r="B10" s="11" t="inlineStr">
+        <is>
+          <t>별도</t>
+        </is>
+      </c>
+      <c r="C10" s="10" t="inlineStr">
+        <is>
+          <t>별도</t>
+        </is>
+      </c>
+      <c r="D10" s="25" t="inlineStr">
+        <is>
+          <t>항목별 내역 없음</t>
+        </is>
+      </c>
+      <c r="E10" s="24" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="11" ht="30" customHeight="1">
+      <c r="A11" s="26" t="inlineStr">
+        <is>
+          <t>합계 (VAT 제외)</t>
+        </is>
+      </c>
+      <c r="B11" s="27" t="inlineStr">
+        <is>
+          <t>230 + α</t>
+        </is>
+      </c>
+      <c r="C11" s="13">
+        <f>C5+C7</f>
+        <v/>
+      </c>
+      <c r="D11" s="13">
+        <f>466094420/1.1/1000000</f>
+        <v/>
+      </c>
+      <c r="E11" s="28">
+        <f>TEXT(230-C11,"+#,##0;-#,##0")&amp;" ("&amp;TEXT(230/C11-1,"+0%;-0%")&amp;")"</f>
+        <v/>
+      </c>
+    </row>
+    <row r="12" ht="30" customHeight="1">
+      <c r="A12" s="26" t="inlineStr">
+        <is>
+          <t>합계 (Optional 포함)</t>
+        </is>
+      </c>
+      <c r="B12" s="27" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="C12" s="13">
+        <f>C11+C8</f>
+        <v/>
+      </c>
+      <c r="D12" s="13">
+        <f>D11</f>
+        <v/>
+      </c>
+      <c r="E12" s="28" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="13" ht="30" customHeight="1">
+      <c r="A13" s="26" t="inlineStr">
+        <is>
+          <t>합계 (VAT 포함)</t>
+        </is>
+      </c>
+      <c r="B13" s="27" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="C13" s="13">
+        <f>C11*1.1</f>
+        <v/>
+      </c>
+      <c r="D13" s="13">
+        <f>466094420/1000000</f>
+        <v/>
+      </c>
+      <c r="E13" s="28" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>• Lihuhu 실제 424 = 제안 ≈283 대비 +50% (Optional 포함 ≈355 대비 +19%)</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>• 결의서 기재 업무는 재무실사·세무실사·가치평가뿐 → 증가 원인 확인 불가 (결의서 첨부 확인 필요)</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>• FDD: Lihuhu 216은 가치평가 포함 → EY FDD 140과 직접 비교 시 차이 과대</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>• TDD: Lihuhu(베트남 1개 법인) ≈67 vs EY 90 → EY가 약 35% 높음 (EY 대상 법인 수 미기재)</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>• EY 230 vs Lihuhu 실제 424 (-46%)이나, EY는 가치평가 미포함 → 범위 차이 감안 필요</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="29" t="inlineStr">
+        <is>
+          <t>※ 실제 466,094,420원 ÷ 1.1 = 423,722,200원 → VAT 포함으로 판단(추정) / 출처: EY 제안서 p.20, Deloitte 제안서(251125) p.27, 지출결의서 20260330-01276</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
   <dimension ref="A1:D10"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
@@ -1518,7 +2189,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -1532,12 +2203,12 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="23" t="inlineStr">
+      <c r="A1" s="30" t="inlineStr">
         <is>
           <t>구분</t>
         </is>
       </c>
-      <c r="B1" s="23" t="inlineStr">
+      <c r="B1" s="30" t="inlineStr">
         <is>
           <t>내용</t>
         </is>

</xml_diff>

<commit_message>
Store calculated values and embed table images in fee workbook
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01MGNZa9FoKJ1mnmQ2XmKaEy
</commit_message>
<xml_diff>
--- a/Scrambly_자문사_보수비교.xlsx
+++ b/Scrambly_자문사_보수비교.xlsx
@@ -274,6 +274,66 @@
     </indexedColors>
   </colors>
 </styleSheet>
+</file>
+
+<file path=xl/drawings/drawing1.xml><?xml version="1.0" encoding="utf-8"?>
+<wsDr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
+  <oneCellAnchor>
+    <from>
+      <col>7</col>
+      <colOff>0</colOff>
+      <row>1</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="7239000" cy="4343400"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="1" name="Image 1" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip cstate="print" r:embed="rId1"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+</wsDr>
+</file>
+
+<file path=xl/drawings/drawing2.xml><?xml version="1.0" encoding="utf-8"?>
+<wsDr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
+  <oneCellAnchor>
+    <from>
+      <col>7</col>
+      <colOff>0</colOff>
+      <row>1</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="7239000" cy="5591175"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="1" name="Image 1" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip cstate="print" r:embed="rId1"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+</wsDr>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -705,14 +765,14 @@
       </c>
       <c r="C10" s="10">
         <f>118000*$B$6/1000000</f>
-        <v/>
+        <v>194.7</v>
       </c>
       <c r="D10" s="9" t="n">
         <v>191</v>
       </c>
       <c r="E10" s="10">
         <f>46000*$B$5/1000000</f>
-        <v/>
+        <v>66.7</v>
       </c>
       <c r="F10" s="10" t="inlineStr">
         <is>
@@ -739,7 +799,7 @@
       </c>
       <c r="C11" s="10">
         <f>20000*$B$6/1000000</f>
-        <v/>
+        <v>33.0</v>
       </c>
       <c r="D11" s="10" t="inlineStr">
         <is>
@@ -748,7 +808,7 @@
       </c>
       <c r="E11" s="10">
         <f>50000*$B$5/1000000</f>
-        <v/>
+        <v>72.5</v>
       </c>
       <c r="F11" s="10" t="inlineStr">
         <is>
@@ -875,23 +935,23 @@
       </c>
       <c r="B15" s="13">
         <f>B9+B10</f>
-        <v/>
+        <v>230.0</v>
       </c>
       <c r="C15" s="13">
         <f>C9+C10</f>
-        <v/>
+        <v>374.7</v>
       </c>
       <c r="D15" s="13">
         <f>SUM(D9:D14)</f>
-        <v/>
+        <v>486.0</v>
       </c>
       <c r="E15" s="13">
         <f>E9+E10</f>
-        <v/>
+        <v>282.7</v>
       </c>
       <c r="F15" s="13">
         <f>466094420/1.1/1000000</f>
-        <v/>
+        <v>423.72219999999993</v>
       </c>
       <c r="G15" s="12" t="inlineStr">
         <is>
@@ -907,23 +967,23 @@
       </c>
       <c r="B16" s="15">
         <f>B15+5</f>
-        <v/>
+        <v>235.0</v>
       </c>
       <c r="C16" s="15">
         <f>C15+C11</f>
-        <v/>
+        <v>407.7</v>
       </c>
       <c r="D16" s="15">
         <f>D15</f>
-        <v/>
+        <v>486.0</v>
       </c>
       <c r="E16" s="15">
         <f>E15+E11</f>
-        <v/>
+        <v>355.2</v>
       </c>
       <c r="F16" s="15">
         <f>F15</f>
-        <v/>
+        <v>423.72219999999993</v>
       </c>
       <c r="G16" s="14" t="inlineStr">
         <is>
@@ -939,23 +999,23 @@
       </c>
       <c r="B17" s="15">
         <f>B15*1.1</f>
-        <v/>
+        <v>253.00000000000003</v>
       </c>
       <c r="C17" s="15">
         <f>C15*1.1</f>
-        <v/>
+        <v>412.17</v>
       </c>
       <c r="D17" s="15">
         <f>D15*1.1</f>
-        <v/>
+        <v>534.6</v>
       </c>
       <c r="E17" s="15">
         <f>E15*1.1</f>
-        <v/>
+        <v>310.97</v>
       </c>
       <c r="F17" s="15">
         <f>466094420/1000000</f>
-        <v/>
+        <v>466.09442</v>
       </c>
       <c r="G17" s="14" t="inlineStr">
         <is>
@@ -973,12 +1033,12 @@
       <c r="C18" s="16" t="inlineStr"/>
       <c r="D18" s="16">
         <f>D15/C15-1</f>
-        <v/>
+        <v>0.29703763010408335</v>
       </c>
       <c r="E18" s="16" t="inlineStr"/>
       <c r="F18" s="16">
         <f>F15/E15-1</f>
-        <v/>
+        <v>0.49884046692606976</v>
       </c>
       <c r="G18" s="14" t="inlineStr">
         <is>
@@ -996,12 +1056,12 @@
       <c r="C19" s="16" t="inlineStr"/>
       <c r="D19" s="16">
         <f>D16/C16-1</f>
-        <v/>
+        <v>0.19205298013245042</v>
       </c>
       <c r="E19" s="16" t="inlineStr"/>
       <c r="F19" s="16">
         <f>F16/E16-1</f>
-        <v/>
+        <v>0.19291159909909883</v>
       </c>
       <c r="G19" s="14" t="inlineStr"/>
     </row>
@@ -1053,19 +1113,19 @@
       </c>
       <c r="B23" s="10">
         <f>B9+B10</f>
-        <v/>
+        <v>230.0</v>
       </c>
       <c r="C23" s="10">
         <f>D9+D10</f>
-        <v/>
+        <v>353.0</v>
       </c>
       <c r="D23" s="10">
         <f>B23-C23</f>
-        <v/>
+        <v>-123.0</v>
       </c>
       <c r="E23" s="19">
         <f>B23/C23-1</f>
-        <v/>
+        <v>-0.3484419263456091</v>
       </c>
       <c r="F23" s="10" t="inlineStr"/>
       <c r="G23" s="18" t="inlineStr">
@@ -1082,19 +1142,19 @@
       </c>
       <c r="B24" s="10">
         <f>B9+B10</f>
-        <v/>
+        <v>230.0</v>
       </c>
       <c r="C24" s="10">
         <f>C9+C10</f>
-        <v/>
+        <v>374.7</v>
       </c>
       <c r="D24" s="10">
         <f>B24-C24</f>
-        <v/>
+        <v>-144.7</v>
       </c>
       <c r="E24" s="19">
         <f>B24/C24-1</f>
-        <v/>
+        <v>-0.3861756071523885</v>
       </c>
       <c r="F24" s="10" t="inlineStr"/>
       <c r="G24" s="18" t="inlineStr"/>
@@ -1107,19 +1167,19 @@
       </c>
       <c r="B25" s="10">
         <f>B9</f>
-        <v/>
+        <v>140.0</v>
       </c>
       <c r="C25" s="10">
         <f>D9</f>
-        <v/>
+        <v>162.0</v>
       </c>
       <c r="D25" s="10">
         <f>B25-C25</f>
-        <v/>
+        <v>-22.0</v>
       </c>
       <c r="E25" s="19">
         <f>B25/C25-1</f>
-        <v/>
+        <v>-0.13580246913580252</v>
       </c>
       <c r="F25" s="10" t="inlineStr"/>
       <c r="G25" s="18" t="inlineStr"/>
@@ -1132,19 +1192,19 @@
       </c>
       <c r="B26" s="10">
         <f>B9</f>
-        <v/>
+        <v>140.0</v>
       </c>
       <c r="C26" s="10">
         <f>C9</f>
-        <v/>
+        <v>180.0</v>
       </c>
       <c r="D26" s="10">
         <f>B26-C26</f>
-        <v/>
+        <v>-40.0</v>
       </c>
       <c r="E26" s="19">
         <f>B26/C26-1</f>
-        <v/>
+        <v>-0.2222222222222222</v>
       </c>
       <c r="F26" s="10" t="inlineStr"/>
       <c r="G26" s="18" t="inlineStr"/>
@@ -1157,19 +1217,19 @@
       </c>
       <c r="B27" s="10">
         <f>B10</f>
-        <v/>
+        <v>90.0</v>
       </c>
       <c r="C27" s="10">
         <f>D10</f>
-        <v/>
+        <v>191.0</v>
       </c>
       <c r="D27" s="10">
         <f>B27-C27</f>
-        <v/>
+        <v>-101.0</v>
       </c>
       <c r="E27" s="19">
         <f>B27/C27-1</f>
-        <v/>
+        <v>-0.5287958115183247</v>
       </c>
       <c r="F27" s="10" t="inlineStr"/>
       <c r="G27" s="18" t="inlineStr">
@@ -1186,19 +1246,19 @@
       </c>
       <c r="B28" s="10">
         <f>B10</f>
-        <v/>
+        <v>90.0</v>
       </c>
       <c r="C28" s="10">
         <f>D10/3</f>
-        <v/>
+        <v>63.666666666666664</v>
       </c>
       <c r="D28" s="10">
         <f>B28-C28</f>
-        <v/>
+        <v>26.333333333333336</v>
       </c>
       <c r="E28" s="19">
         <f>B28/C28-1</f>
-        <v/>
+        <v>0.4136125654450262</v>
       </c>
       <c r="F28" s="10" t="inlineStr"/>
       <c r="G28" s="18" t="inlineStr">
@@ -1215,19 +1275,19 @@
       </c>
       <c r="B29" s="10">
         <f>B10</f>
-        <v/>
+        <v>90.0</v>
       </c>
       <c r="C29" s="10">
         <f>E10</f>
-        <v/>
+        <v>66.7</v>
       </c>
       <c r="D29" s="10">
         <f>B29-C29</f>
-        <v/>
+        <v>23.299999999999997</v>
       </c>
       <c r="E29" s="19">
         <f>B29/C29-1</f>
-        <v/>
+        <v>0.3493253373313343</v>
       </c>
       <c r="F29" s="10" t="inlineStr"/>
       <c r="G29" s="18" t="inlineStr">
@@ -1251,7 +1311,7 @@
       </c>
       <c r="B32" s="9">
         <f>B15</f>
-        <v/>
+        <v>230.0</v>
       </c>
     </row>
     <row r="33">
@@ -1272,7 +1332,7 @@
       </c>
       <c r="B34" s="9">
         <f>0*504*$B$6/1000000</f>
-        <v/>
+        <v>0.0</v>
       </c>
       <c r="C34" s="5" t="inlineStr">
         <is>
@@ -1298,7 +1358,7 @@
       </c>
       <c r="B36" s="22">
         <f>SUM(B32:B35)</f>
-        <v/>
+        <v>241.0</v>
       </c>
     </row>
     <row r="37">
@@ -1309,7 +1369,7 @@
       </c>
       <c r="B37" s="22">
         <f>B36*1.1</f>
-        <v/>
+        <v>265.1</v>
       </c>
     </row>
   </sheetData>
@@ -1323,7 +1383,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E20"/>
+  <dimension ref="A1:H20"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="24" customWidth="1" min="1" max="1"/>
@@ -1340,6 +1400,11 @@
           <t>[Scrambly] 실사 자문 보수 비교 – EY 제안 vs Deloitte JustPlay</t>
         </is>
       </c>
+      <c r="H1" s="3" t="inlineStr">
+        <is>
+          <t>Teams 첨부용 표 이미지</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
@@ -1393,9 +1458,9 @@
       <c r="D5" s="10" t="n">
         <v>162</v>
       </c>
-      <c r="E5" s="24">
+      <c r="E5" s="24" t="str">
         <f>TEXT(B5-D5,"+#,##0;-#,##0")&amp;" ("&amp;TEXT(B5/D5-1,"+0%;-0%")&amp;")"</f>
-        <v/>
+        <v>-22 (-14%)</v>
       </c>
     </row>
     <row r="6" ht="30" customHeight="1">
@@ -1409,14 +1474,14 @@
       </c>
       <c r="C6" s="10">
         <f>118000*비교표!$B$6/1000000</f>
-        <v/>
+        <v>194.7</v>
       </c>
       <c r="D6" s="10" t="n">
         <v>191</v>
       </c>
-      <c r="E6" s="24">
+      <c r="E6" s="24" t="str">
         <f>TEXT(B6-D6,"+#,##0;-#,##0")&amp;" ("&amp;TEXT(B6/D6-1,"+0%;-0%")&amp;")"</f>
-        <v/>
+        <v>-101 (-53%)</v>
       </c>
     </row>
     <row r="7" ht="30" customHeight="1">
@@ -1432,7 +1497,7 @@
       </c>
       <c r="C7" s="10">
         <f>20000*비교표!$B$6/1000000</f>
-        <v/>
+        <v>33.0</v>
       </c>
       <c r="D7" s="25" t="inlineStr">
         <is>
@@ -1533,11 +1598,11 @@
       </c>
       <c r="C11" s="13">
         <f>C5+C6</f>
-        <v/>
+        <v>374.7</v>
       </c>
       <c r="D11" s="13">
         <f>SUM(D5:D10)</f>
-        <v/>
+        <v>486.0</v>
       </c>
       <c r="E11" s="28" t="inlineStr">
         <is>
@@ -1553,19 +1618,19 @@
       </c>
       <c r="B12" s="27">
         <f>B5+B6</f>
-        <v/>
+        <v>230.0</v>
       </c>
       <c r="C12" s="13">
         <f>C5+C6</f>
-        <v/>
+        <v>374.7</v>
       </c>
       <c r="D12" s="13">
         <f>D5+D6</f>
-        <v/>
-      </c>
-      <c r="E12" s="28">
+        <v>353.0</v>
+      </c>
+      <c r="E12" s="28" t="str">
         <f>TEXT(B12-D12,"+#,##0;-#,##0")&amp;" ("&amp;TEXT(B12/D12-1,"+0%;-0%")&amp;")"</f>
-        <v/>
+        <v>-123 (-35%)</v>
       </c>
     </row>
     <row r="14">
@@ -1612,6 +1677,7 @@
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
 </worksheet>
 </file>
 
@@ -1621,7 +1687,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E21"/>
+  <dimension ref="A1:H21"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="24" customWidth="1" min="1" max="1"/>
@@ -1638,6 +1704,11 @@
           <t>[Scrambly] 실사 자문 보수 비교 – EY 제안 vs Deloitte Lihuhu</t>
         </is>
       </c>
+      <c r="H1" s="3" t="inlineStr">
+        <is>
+          <t>Teams 첨부용 표 이미지</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
@@ -1693,9 +1764,9 @@
           <t>항목별 내역 없음</t>
         </is>
       </c>
-      <c r="E5" s="24">
+      <c r="E5" s="24" t="str">
         <f>TEXT(B5-C5,"+#,##0;-#,##0")&amp;" ("&amp;TEXT(B5/C5-1,"+0%;-0%")&amp;")"&amp;" *가치평가 포함"</f>
-        <v/>
+        <v>-76 (-35%) *가치평가 포함</v>
       </c>
     </row>
     <row r="6" ht="30" customHeight="1">
@@ -1736,16 +1807,16 @@
       </c>
       <c r="C7" s="10">
         <f>46000*비교표!$B$5/1000000</f>
-        <v/>
+        <v>66.7</v>
       </c>
       <c r="D7" s="25" t="inlineStr">
         <is>
           <t>항목별 내역 없음</t>
         </is>
       </c>
-      <c r="E7" s="24">
+      <c r="E7" s="24" t="str">
         <f>TEXT(B7-C7,"+#,##0;-#,##0")&amp;" ("&amp;TEXT(B7/C7-1,"+0%;-0%")&amp;")"</f>
-        <v/>
+        <v>+23 (+35%)</v>
       </c>
     </row>
     <row r="8" ht="30" customHeight="1">
@@ -1761,7 +1832,7 @@
       </c>
       <c r="C8" s="10">
         <f>50000*비교표!$B$5/1000000</f>
-        <v/>
+        <v>72.5</v>
       </c>
       <c r="D8" s="25" t="inlineStr">
         <is>
@@ -1841,15 +1912,15 @@
       </c>
       <c r="C11" s="13">
         <f>C5+C7</f>
-        <v/>
+        <v>282.7</v>
       </c>
       <c r="D11" s="13">
         <f>466094420/1.1/1000000</f>
-        <v/>
-      </c>
-      <c r="E11" s="28">
+        <v>423.72219999999993</v>
+      </c>
+      <c r="E11" s="28" t="str">
         <f>TEXT(230-C11,"+#,##0;-#,##0")&amp;" ("&amp;TEXT(230/C11-1,"+0%;-0%")&amp;")"</f>
-        <v/>
+        <v>-53 (-19%)</v>
       </c>
     </row>
     <row r="12" ht="30" customHeight="1">
@@ -1865,11 +1936,11 @@
       </c>
       <c r="C12" s="13">
         <f>C11+C8</f>
-        <v/>
+        <v>355.2</v>
       </c>
       <c r="D12" s="13">
         <f>D11</f>
-        <v/>
+        <v>423.72219999999993</v>
       </c>
       <c r="E12" s="28" t="inlineStr">
         <is>
@@ -1890,11 +1961,11 @@
       </c>
       <c r="C13" s="13">
         <f>C11*1.1</f>
-        <v/>
+        <v>310.97</v>
       </c>
       <c r="D13" s="13">
         <f>466094420/1000000</f>
-        <v/>
+        <v>466.09442</v>
       </c>
       <c r="E13" s="28" t="inlineStr">
         <is>
@@ -1946,6 +2017,7 @@
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
 </worksheet>
 </file>
 

</xml_diff>